<commit_message>
Audyt 30.09: raport zbiorczy + arkusz (8 arkuszy) + 3 raporty szczegółowe (Routines, spójność strony, teksty szablonowe)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011GrNNd6UVQFF1NamoPaQMS
</commit_message>
<xml_diff>
--- a/materialy/audyt-2026-09-30.xlsx
+++ b/materialy/audyt-2026-09-30.xlsx
@@ -9,9 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Afiliacje" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Źródła danych" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cloudflare" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firecrawl" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indeksacja (GSC)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routines (co-kto-kiedy-status)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cloudflare" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firecrawl" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indeksacja (GSC)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strona — top 10" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teksty — top 10" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2388,6 +2391,583 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Co robi</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Kto (nazwa · sesja · model)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Kiedy (cron UTC → PL)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status (last_run · commit)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Wejście</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Wyjście</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Dogrywa do R2 zdjęcia, których worker sam nie pobierze (od 27.09 wszystkie źródła)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>„LEGO 04:30 — Zdjęcia → R2" · świeża sesja (z panelu), 6 konektorów, bez repo w źródłach · model domyślny</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>`30 2 * * *` → codziennie 04:30 (dryf do 04:40)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>✅ 30.09 04:40, 47 s · bez commitów z założenia</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>`obrazy.json`, `galerie.json`, `zdjecia.json`; `CF_R2_TOKEN`</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>kubełek R2 `tylkoklocki-obrazy`, ślad `_stan/r2-obrazy.json`</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Nowości i przecieki: Brickset/PromoBricks/StoneWars → nowe sety, luki katalogu, sygnały wycofań do DZIENNIKA</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>„LEGO 05:00 — Scout nowości" · trwała `session_012AZejbFzsfzkTh4FPaAkVg` · Opus 5</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>`0 3 * * *` → codziennie 05:00</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>✅ 30.09 05:04 · commity 22, 23, 24, 25, 26, **(27, 28 brak — weekend, „bez nowości")**, 29, 30.09 (30.09 05:07 i 05:08)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Brickset, PromoBricks, StoneWars; `known_sets.json`, `oferty_feed.json` (luki)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>`sety.json`, `known_sets.json`, `przecieki.json`, wpis SCOUT w `DZIENNIK.md`; mail `nowosci` (Resend) gdy był commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Tygodniowy zaciąg listingu lego.pl (Firecrawl, ~75 kredytów) + RRP + linki LEGO + Rebrickable + Ceneo/Lidl (TD) + Smyk</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>„Dane wt 05:30 — katalog LEGO.pl + ceny Ceneo i Smyk" · trwała `session_011Ced7USAHUBBsCPZ1os3F9` · Sonnet 5 (co-author commita)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>`30 3 * * 2` → wtorek 05:30 (dryf 05:34)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>✅ 29.09 05:34 · **commit 0c2d3fc 29.09 05:52 PL z tej sesji** — pierwszy prawdziwy przebieg runnera zaliczony; UWAGA: tytuł commita skopiowany z 22.09 i mówi „(sesja Code za runnera)", co jest nieprawdą</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>`FIRECRAWL_KEY`, `TD_TOKEN`; `feedy.json`, `redirects.smyk`</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>`oferty_feed.json` (`lego`, `ceneo`, `lidl`, `smyk`), `sety.json`, `katalog.json` (status/ekskluzyw/`lego_pl_widziano`/nowe z Rebrickable), `rrp_potwierdzone.json`, `redirects.json` (`lego`, `ceneo`, `lidl`), `obrazy.json`; build</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Wycofania: lego.com „Ostatnie sztuki", Brickset, StoneWars/PromoBricks + sygnały Scouta</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>„LEGO pon 06:10 — Wycofania" · trwała `session_01KfWF14fJvwK78sBVG6XAz8` · Fable 5</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>`10 4 * * 1` → pon 06:10</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>✅ 28.09 06:10 · commit 644240f 28.09 06:14 PL; **21.09 bez commita** (nic się nie zmieniło? — prompt pozwala nie commitować; nie zweryfikowano)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>źródła www, `DZIENNIK.md` (SCOUT), `katalog.json` (tylko odczyt)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>`wycofania.json` (jedyny autor), adnotacje `→ Wycofania` w `DZIENNIK.md`; `audyt-wycofan.mjs` raport; mail `wycofania`</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Przepisuje harmonogram i prompty z konta do repo (`list_triggers`)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>„LEGO pon 07:45 — Harmonogram z konta" · trwała sesja Code `session_01XzZ5hRoRbmYj4cURMXc2ES` (**nie ta bieżąca**) · sesja Code</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>`45 5 * * 1` → pon 07:45</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>✅ 28.09 07:45 · commit 3023be7 28.09 07:47 PL</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>`list_triggers` (jedyna sesja z konektorem `Claude_Code_Remote`)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>`materialy/zadania-cykliczne.md` (sekcja Zrzut), `materialy/routine-prompty.md`</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Radar konkurencji: fanklockow, faniklockow, zklockow, promoklocki (+ klockoradar wg `_meta`)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>„LEGO 08:00 — Radar konkurencji" · trwała `session_01UFkqKNwQexnxLN34HotM4G` · Opus 5</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>`0 6 * * *` → codziennie 08:00 (dryf 08:17)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>✅ 30.09 08:17 · commity codziennie 22–30.09 (9/9)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>strony konkurencji, `konkurencja_baza.json`</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>`konkurencja_baza.json`, wpis „RADAR · Do zrobienia" w `DZIENNIK.md`; mail `konkurencja` gdy commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Uruchamia skill zrzutu Empiku w chmurze</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>„Empik co tydzien" · świeża sesja (z panelu, `permission_mode: auto`), 7 konektorów (w tym `Claude_Code_Remote`, Firecrawl) · model domyślny</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>`CRON_TZ=Europe/Warsaw 0 8 * * 1` → pon 08:00 (dryf 08:11; 28.09 odpalił 08:59)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>✅ 28.09 08:59–09:21 (22 min) · **żaden artefakt**: dane Empiku z 28.09 (a460501 08:56 PL) pochodzą z pliku od Marka wgranego do sesji Code 08:40, czyli PRZED startem tego Routine</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>prompt: `uruchom skill: klocki-ceny-empik` (skill wymaga lokalnej przeglądarki; Empik daje 403 z chmury, Playwright w kontenerze = ERR_CONNECTION_RESET)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>nic sprawdzalnego; 22 min limitu konta co poniedziałek</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Mail-przypominajka o ręcznym zrzucie Empiku</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>„LEGO pon 08:15 — Przypomnienie: zrzut Empiku" · świeża sesja (z panelu) · model domyślny</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>`15 6 * * 1` → pon 08:15</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>✅ 28.09 08:16, 81 s · bez commitów z założenia</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>`RESEND_API_KEY`, `raporty_mail.json` (`przypomnienie`)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>1 mail na kontakt@</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Ceny z feedów ME/PK/Allegro (+ Lidl codziennie, Smyk w piątki, kontrola linków w poniedziałki, historia cen), deale, posty dealowe, mail „podejrzany rynek"</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>„LEGO 08:30 — Łowca promocji" · trwała `session_01SdxKtAvW8UmktsuXrsPYga` (od 22.09) · Fable 5</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>`30 6 * * *` → codziennie 08:30 (dryf 08:41)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>✅ 29.09 08:42 (30.09 jeszcze przed slotem w chwili odczytu) · commity codziennie 22–29.09 (8/8), commit ląduje 08:58–09:15 PL; 28.09 dodatkowy commit 45acf8f „odzyskane 732 wpisy historii cen" po zderzeniu z importem Empiku</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>`feedy-lego.py` (feedy ME/PK/Allegro/TD), `ceny_baza.json`, `wycofania.json`, opcjonalnie `lego-empik.json`</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>`oferty_feed.json` (`mediaexpert`, `planetaklockow`, `allegro`, `lidl`, pt `smyk`), `ceny_baza.json`, `redirects.json` (PK, allegro, ME, lidl), `sety.json`, `obrazy.json`, `src/pages/deale/*.md`, `historia-cen/RRRR-MM.jsonl`, pon `materialy/kontrola-linkow-*.md`; maile `promocje` (zawsze), `podejrzane`, `linki`</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Raport tygodnia: diagnoza, kliki, prowizje, GSC, indeksacja, harmonogram (czyta), archiwum dziennika, „zadania bez właściciela"</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>„LEGO pon 09:00 — Kontroler" · trwała `session_01M8qMJFfKHEozBSGXjAKP4n` · Opus 5</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>`0 7 * * 1` → pon 09:00 (dryf 09:21)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>✅ 28.09 09:21 · commit 37258ab 28.09 09:35 PL (raport + archiwum 8 wpisów); 22.09 przebieg próbny</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>`diagnoza.mjs`, `kliki-raport.mjs`, `prowizje-raport.mjs`, `gsc-raport.mjs`, GSC URL Inspection, `materialy/kontrola-linkow-*.md`, `DZIENNIK.md`, build</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>`materialy/kontroler-RRRR-MM-DD.md`, `DZIENNIK.md` + `materialy/dziennik-archiwum-*.md`; PDF przez SendUserFile; mail `kontroler` (Marek + Piotr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Alerty „Obserwuj zestaw": porównuje ceny z repo z progiem, wysyła maile, kasuje niepotwierdzone zapisy</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>„LEGO 09:30 — Alerty cen" · świeża sesja (z panelu) · model domyślny</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>`30 7 * * *` → codziennie 09:30 (dryf 09:34–09:36)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>✅ 29.09 09:36, 26 s · bez commitów z założenia</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>R2 `_obserwuj/`, `oferty_feed.json`/`sety.json` z klonu `--depth 1`; `CF_R2_TOKEN`, `RESEND_API_KEY`</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>maile do czytelników; kasowanie obiektów w R2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Backfill cen katalogowych z Brickset/promoklocki</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>„LEGO co 8h — Backfill cen katalogowych" · trwała `session_01JSfUBJxddBbATeaXhQ6efS` · Fable 5</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>`0 2,10,18 * * *` → 04/12/20</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>❌ **wyłączony**, nigdy nie odpalony pod tym ID (odtworzony 31.08)</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>`katalog.json`, Brickset/promoklocki</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>`katalog.json.cena_katalogowa` — dziś nikt</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Jednorazowo: czy `/promocje-lego/`, `/` i `/deale/` (301) są w indeksie po wdrożeniu 29.09</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>„GSC: czy /promocje-lego/ w indeksie" · przypięty do bieżącej sesji Code `session_011GrNNd6UVQFF1NamoPaQMS`</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>`run_once_at` 02.10 08:52 PL</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>⏳ czeka</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>GSC URL Inspection (`GSC_KEY_JSON_B64`)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>linia w `DZIENNIK.md` (wpis 29.09 12:40), push</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Jednorazowo: raport kliknięć 14 dni po CRO (odniesienie: 139 klików / 14 dni z 25.09)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>„Raport kliknięć — skutek CRO" · bieżąca sesja Code</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>`run_once_at` 09.10 09:00 PL</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>⏳ czeka</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>`kliki-raport.mjs --dni 14`</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>tabela przed/po, „→ zamknięte" w `DZIENNIK.md`, push</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3134,7 +3714,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3357,7 +3937,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3767,4 +4347,192 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Do naprawy (wg wpływu na czytelnika i Google) — pełny raport: materialy/audyt-2026-09-30/strona-spojnosc.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>**Meta description &gt; 160 zn. na 1 300 indeksowalnych stron** (1 239 hubów, 33 artykuły) —</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>**Title &gt; 60 zn. na 1 241 indeksowalnych** (huby mediana 75) — skrócić wzorzec tytułu huba</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>**Pozostałości `/podglad/deale-obecne/`, `/podglad/glowna-obecna/`** żyją na produkcji (200) —</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>**`/polityka-prywatnosci/` bez linku w stopce i poza sitemapą** — `Base.astro` (stopka) +</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>**`/nowosci/` (12 stron): h1 → h3** — `src/pages/nowosci/[miesiac].astro` L148 i `nowosci.astro` → `&lt;h2&gt;`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>**`/kolekcjoner/` – sierota-stub** (0 linków, noindex) — usunąć albo 301 → `/wycofania/` w `public/_redirects`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>**Brak JSON-LD (nawet BreadcrumbList) na listingach** `/artykuly/`, `/promocje-lego/`, `/nowosci/`,</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>**Zestawy GWP z wierszem „LEGO.com &lt;cena przypisana&gt;" jako ofertą** (`/zestaw/40896/`; LD low ≠ tabela) —</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>**Stopkowe `&lt;h4&gt;` łamią hierarchię na każdej stronie** (h2→h4, na 15 stronach h1→h4) — `Base.astro`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>**Drobiazgi hubów**: 2 huby z tabelą zawierającą tylko „produkcja zakończona" bez CTA (`2198, 7235`) →</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Do poprawy w tekstach szablonowych — pełny raport: materialy/audyt-2026-09-30/teksty-szablonowe.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>**Wyciąć z `opisy.json` zdania o dostępności i rynku wtórnym** (ok. 9 tys. zdań: „dziś dostępny głównie z drugiej ręki”, „krąży po rynku wtórnym w rozsądnych cenach”, „Aktualnie w sprzedaży – ceny sprawdzamy codziennie rano”, „Nie ma go już w śledzonych sklepach”). Stoją obok żywej tabeli i jej przeczą na /promocje-lego/, w tabelach serii i wycofań – najbardziej widoczny dowód, że tekst pisze maszyna. Zostawić tylko rozmiar + rocznik, bez „wyraźnie kolekcjonerski” i „Klasyk”.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>**Warunkowa meta description huba** (`[nr].astro:203–219`): „dla rodzica i dla kolekcjonera” tylko gdy persony są, „rabat od RRP” tylko gdy jest RRP, dla EOL osobne zdanie zamiast „promocji jeszcze nie ma – sprawdzamy codziennie”. Dotyczy 4–5 tys. snippetów w Google.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>**Jedna nota afiliacyjna** (brzmienie z `Base.astro:198`) w Artykul, PrezentownikSerii, hubie i trzech listingach; jedno zdanie o koszyku pod tabelą zamiast dwóch; wyciąć „Różnica zwykle wypada na Twoją korzyść”.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>**Funkcja odmiany liczebnika** w `src/lib/oferty.js` (wzór: `odmienZestaw` z `serie-listing.js`) i użycie w 10 miejscach: elementów, zestawów, ofert, zdjęć, trafień, prognoz, pozycji, przecieków, zapowiedzi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>**„cena katalogowa nieogłoszona (podamy, gdy LEGO ją poda)”** → tylko dla zapowiedzi; dla roczników ≤2025 „brak w naszych danych” (`[nr].astro:286, 353`; 4882 hubów).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>**„Ostatnie sztuki w sklepach” / „zapasy” tylko gdy jest sklep z własnym magazynem**; przy samym Allegro „rynek wtórny” (`[nr].astro:150, 303`; 1640 hubów).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>**`akapity_redakcyjne`: rocznik = rok premiery zestawu**, a nie 2026; pomijać akapit dla zestawów starszych niż 3 lata; wyciąć zdanie „Różnią się charakterem…” (`import-karty.py:253–277`; 228 kart z fałszywym porównaniem).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>**`linkuj`: link z placeholdera jako pełne zdanie** z wielką literą i kropką („Bieżące ceny są w tabeli wyżej.”), jedna forma zamiast trzech (`import-karty.py:187–192`; 882 hubów).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>**/wycofania/**: liczba serii z danych zamiast „w 11 seriach”, lead skrócony do 4 zdań, bez „Wracaj tu regularnie” ×2 i bez „kup przed zniknięciem, po EOL ceny rosną” (sprzeczne z własnym FAQ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>**Obietnica „codziennie”** – zostawić tylko tam, gdzie prawdziwa (Łowca: Media Expert, Planeta, Allegro, Empik), a w hubach z samym LEGO.com/Ceneo/Smyk i w 17 stopkach prezentowników zastąpić „w dni robocze” / usunąć; „w historii” → „w naszych notowaniach”. Do tego: `{?}` w H2 karty (4 huby, `[nr].astro:390`), „premiera 2021-01” → „styczeń 2021” (`[nr].astro:281`), „wycofanie w XII 2026” z danych (`KartaPrezentu.astro:78`), „Każda cena z datą sprawdzenia” (`prezentowniki.astro:53`) – małe, ale rzucają się w oczy.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>